<commit_message>
Remove leftover n8n director code and keep Q&A on the local Python director.
The live talk path already lives in this app, so the unused workflow, Docker stack, and n8n-specific UI only added confusion.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/knowledge_sources/knowledge.xlsx
+++ b/data/knowledge_sources/knowledge.xlsx
@@ -583,17 +583,17 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Presenter,產品,粵語,跟稿,n8n,簡報代理,product</t>
+          <t>Presenter,產品,粵語,跟稿,導演,簡報代理,product,director</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Harbour Presenter 係粵語優先語音簡報代理，跟預先寫好嘅稿講，唔即場生稿。n8n 做導演，PowerPoint 跟住翻頁。呢頁就係產品頁。</t>
+          <t>Harbour Presenter 係粵語優先語音簡報代理，跟預先寫好嘅稿講，唔即場生稿。本機導演控制節奏，PowerPoint 跟住翻頁。呢頁就係產品頁。</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Harbour Presenter is a Cantonese-first voice presenter that reads a prepared script. n8n directs; PowerPoint follows. That is the product slide.</t>
+          <t>Harbour Presenter is a Cantonese-first voice presenter that reads a prepared script. The local director controls pacing; PowerPoint follows. That is the product slide.</t>
         </is>
       </c>
     </row>

</xml_diff>